<commit_message>
Drag-and-drop manual level lines on the chart
- N-SL / N-TP lines on the NIFTY chart are now draggable: hover shows
  ns-resize cursor, mousedown grabs the line (chart pan/zoom suspended),
  the line follows the mouse live, release sends set_manual_levels
- Server validates side-correctness; an invalid drop snaps the line back
  via the state echo; broadcasts never yank a line mid-drag (2s hold
  window after release for the round-trip)
- Numeric inputs in the Scalp panel kept as a precision fallback
- Verified headless: synthetic drag moved SL 24020.4 -> 24009.4 and
  emitted the update; pan restored after release; zero JS errors

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trade_log.xlsx
+++ b/trade_log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2468,6 +2468,73 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>12:47:19</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>NIFTY2671424000CE</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>158</v>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>159.15</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>672.75</v>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>nifty_tp</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>279</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>100672.75</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>